<commit_message>
corrigindo o bug de hierarquia dos notebooks de normalização e atualizando os outputs
</commit_message>
<xml_diff>
--- a/02-Referencias/ATUA/ATUA_despesas_fechamento_03-2026.xlsx
+++ b/02-Referencias/ATUA/ATUA_despesas_fechamento_03-2026.xlsx
@@ -608,42 +608,42 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>DESPESA</t>
+          <t>TRANSMOVE GSL</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>1.4 DESPESA</t>
+          <t>1.4 TRANSMOVE GSL</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>1.4</t>
+          <t>1.4.2</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>TRANSMOVE GSL</t>
+          <t>DOURADOS</t>
         </is>
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>1.4 TRANSMOVE GSL</t>
+          <t>1.4.2 DOURADOS</t>
         </is>
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>1.4.2</t>
+          <t>1.4.2.2</t>
         </is>
       </c>
       <c r="J2" t="inlineStr">
         <is>
-          <t>DOURADOS</t>
+          <t>ADMINISTRATIVO</t>
         </is>
       </c>
       <c r="K2" t="inlineStr">
         <is>
-          <t>1.4.2 DOURADOS</t>
+          <t>1.4.2.2 ADMINISTRATIVO</t>
         </is>
       </c>
       <c r="L2" t="inlineStr">
@@ -754,42 +754,42 @@
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>DESPESA</t>
+          <t>TRANSMOVE GSL</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>1.4 DESPESA</t>
+          <t>1.4 TRANSMOVE GSL</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>1.4</t>
+          <t>1.4.1</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>TRANSMOVE GSL</t>
+          <t>PRESIDENTE PRUDENTE</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>1.4 TRANSMOVE GSL</t>
+          <t>1.4.1 PRESIDENTE PRUDENTE</t>
         </is>
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>1.4.1</t>
+          <t>1.4.1.2</t>
         </is>
       </c>
       <c r="J3" t="inlineStr">
         <is>
-          <t>PRESIDENTE PRUDENTE</t>
+          <t>ADMINISTRATIVO</t>
         </is>
       </c>
       <c r="K3" t="inlineStr">
         <is>
-          <t>1.4.1 PRESIDENTE PRUDENTE</t>
+          <t>1.4.1.2 ADMINISTRATIVO</t>
         </is>
       </c>
       <c r="L3" t="inlineStr">
@@ -900,42 +900,42 @@
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>DESPESA</t>
+          <t>TRANSMOVE GSL</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>1.4 DESPESA</t>
+          <t>1.4 TRANSMOVE GSL</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>1.4</t>
+          <t>1.4.1</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>TRANSMOVE GSL</t>
+          <t>PRESIDENTE PRUDENTE</t>
         </is>
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>1.4 TRANSMOVE GSL</t>
+          <t>1.4.1 PRESIDENTE PRUDENTE</t>
         </is>
       </c>
       <c r="I4" t="inlineStr">
         <is>
-          <t>1.4.1</t>
+          <t>1.4.1.1</t>
         </is>
       </c>
       <c r="J4" t="inlineStr">
         <is>
-          <t>PRESIDENTE PRUDENTE</t>
+          <t>TRANSPORTE</t>
         </is>
       </c>
       <c r="K4" t="inlineStr">
         <is>
-          <t>1.4.1 PRESIDENTE PRUDENTE</t>
+          <t>1.4.1.1 TRANSPORTE</t>
         </is>
       </c>
       <c r="L4" t="inlineStr">
@@ -1046,42 +1046,42 @@
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>DESPESA</t>
+          <t>TRANSMOVE GSL</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>1.4 DESPESA</t>
+          <t>1.4 TRANSMOVE GSL</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>1.4</t>
+          <t>1.4.1</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>TRANSMOVE GSL</t>
+          <t>PRESIDENTE PRUDENTE</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>1.4 TRANSMOVE GSL</t>
+          <t>1.4.1 PRESIDENTE PRUDENTE</t>
         </is>
       </c>
       <c r="I5" t="inlineStr">
         <is>
-          <t>1.4.1</t>
+          <t>1.4.1.1</t>
         </is>
       </c>
       <c r="J5" t="inlineStr">
         <is>
-          <t>PRESIDENTE PRUDENTE</t>
+          <t>TRANSPORTE</t>
         </is>
       </c>
       <c r="K5" t="inlineStr">
         <is>
-          <t>1.4.1 PRESIDENTE PRUDENTE</t>
+          <t>1.4.1.1 TRANSPORTE</t>
         </is>
       </c>
       <c r="L5" t="inlineStr">
@@ -1192,42 +1192,42 @@
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>DESPESA</t>
+          <t>TRANSMOVE GSL</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>1.4 DESPESA</t>
+          <t>1.4 TRANSMOVE GSL</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>1.4</t>
+          <t>1.4.1</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>TRANSMOVE GSL</t>
+          <t>PRESIDENTE PRUDENTE</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>1.4 TRANSMOVE GSL</t>
+          <t>1.4.1 PRESIDENTE PRUDENTE</t>
         </is>
       </c>
       <c r="I6" t="inlineStr">
         <is>
-          <t>1.4.1</t>
+          <t>1.4.1.1</t>
         </is>
       </c>
       <c r="J6" t="inlineStr">
         <is>
-          <t>PRESIDENTE PRUDENTE</t>
+          <t>TRANSPORTE</t>
         </is>
       </c>
       <c r="K6" t="inlineStr">
         <is>
-          <t>1.4.1 PRESIDENTE PRUDENTE</t>
+          <t>1.4.1.1 TRANSPORTE</t>
         </is>
       </c>
       <c r="L6" t="inlineStr">
@@ -1338,42 +1338,42 @@
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>DESPESA</t>
+          <t>TRANSMOVE GSL</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>1.4 DESPESA</t>
+          <t>1.4 TRANSMOVE GSL</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>1.4</t>
+          <t>1.4.1</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>TRANSMOVE GSL</t>
+          <t>PRESIDENTE PRUDENTE</t>
         </is>
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>1.4 TRANSMOVE GSL</t>
+          <t>1.4.1 PRESIDENTE PRUDENTE</t>
         </is>
       </c>
       <c r="I7" t="inlineStr">
         <is>
-          <t>1.4.1</t>
+          <t>1.4.1.1</t>
         </is>
       </c>
       <c r="J7" t="inlineStr">
         <is>
-          <t>PRESIDENTE PRUDENTE</t>
+          <t>TRANSPORTE</t>
         </is>
       </c>
       <c r="K7" t="inlineStr">
         <is>
-          <t>1.4.1 PRESIDENTE PRUDENTE</t>
+          <t>1.4.1.1 TRANSPORTE</t>
         </is>
       </c>
       <c r="L7" t="inlineStr">
@@ -1484,42 +1484,42 @@
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>DESPESA</t>
+          <t>TRANSMOVE GSL</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>1.4 DESPESA</t>
+          <t>1.4 TRANSMOVE GSL</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>1.4</t>
+          <t>1.4.1</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>TRANSMOVE GSL</t>
+          <t>PRESIDENTE PRUDENTE</t>
         </is>
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>1.4 TRANSMOVE GSL</t>
+          <t>1.4.1 PRESIDENTE PRUDENTE</t>
         </is>
       </c>
       <c r="I8" t="inlineStr">
         <is>
-          <t>1.4.1</t>
+          <t>1.4.1.2</t>
         </is>
       </c>
       <c r="J8" t="inlineStr">
         <is>
-          <t>PRESIDENTE PRUDENTE</t>
+          <t>ADMINISTRATIVO</t>
         </is>
       </c>
       <c r="K8" t="inlineStr">
         <is>
-          <t>1.4.1 PRESIDENTE PRUDENTE</t>
+          <t>1.4.1.2 ADMINISTRATIVO</t>
         </is>
       </c>
       <c r="L8" t="inlineStr">
@@ -1630,42 +1630,42 @@
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>DESPESA</t>
+          <t>TRANSMOVE GSL</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>1.4 DESPESA</t>
+          <t>1.4 TRANSMOVE GSL</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>1.4</t>
+          <t>1.4.1</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>TRANSMOVE GSL</t>
+          <t>PRESIDENTE PRUDENTE</t>
         </is>
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>1.4 TRANSMOVE GSL</t>
+          <t>1.4.1 PRESIDENTE PRUDENTE</t>
         </is>
       </c>
       <c r="I9" t="inlineStr">
         <is>
-          <t>1.4.1</t>
+          <t>1.4.1.1</t>
         </is>
       </c>
       <c r="J9" t="inlineStr">
         <is>
-          <t>PRESIDENTE PRUDENTE</t>
+          <t>TRANSPORTE</t>
         </is>
       </c>
       <c r="K9" t="inlineStr">
         <is>
-          <t>1.4.1 PRESIDENTE PRUDENTE</t>
+          <t>1.4.1.1 TRANSPORTE</t>
         </is>
       </c>
       <c r="L9" t="inlineStr">
@@ -1776,42 +1776,42 @@
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>DESPESA</t>
+          <t>TRANSMOVE GSL</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>1.4 DESPESA</t>
+          <t>1.4 TRANSMOVE GSL</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>1.4</t>
+          <t>1.4.1</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>TRANSMOVE GSL</t>
+          <t>PRESIDENTE PRUDENTE</t>
         </is>
       </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t>1.4 TRANSMOVE GSL</t>
+          <t>1.4.1 PRESIDENTE PRUDENTE</t>
         </is>
       </c>
       <c r="I10" t="inlineStr">
         <is>
-          <t>1.4.1</t>
+          <t>1.4.1.1</t>
         </is>
       </c>
       <c r="J10" t="inlineStr">
         <is>
-          <t>PRESIDENTE PRUDENTE</t>
+          <t>TRANSPORTE</t>
         </is>
       </c>
       <c r="K10" t="inlineStr">
         <is>
-          <t>1.4.1 PRESIDENTE PRUDENTE</t>
+          <t>1.4.1.1 TRANSPORTE</t>
         </is>
       </c>
       <c r="L10" t="inlineStr">
@@ -1922,42 +1922,42 @@
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>DESPESA</t>
+          <t>TRANSMOVE GSL</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>1.4 DESPESA</t>
+          <t>1.4 TRANSMOVE GSL</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>1.4</t>
+          <t>1.4.1</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>TRANSMOVE GSL</t>
+          <t>PRESIDENTE PRUDENTE</t>
         </is>
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>1.4 TRANSMOVE GSL</t>
+          <t>1.4.1 PRESIDENTE PRUDENTE</t>
         </is>
       </c>
       <c r="I11" t="inlineStr">
         <is>
-          <t>1.4.1</t>
+          <t>1.4.1.2</t>
         </is>
       </c>
       <c r="J11" t="inlineStr">
         <is>
-          <t>PRESIDENTE PRUDENTE</t>
+          <t>ADMINISTRATIVO</t>
         </is>
       </c>
       <c r="K11" t="inlineStr">
         <is>
-          <t>1.4.1 PRESIDENTE PRUDENTE</t>
+          <t>1.4.1.2 ADMINISTRATIVO</t>
         </is>
       </c>
       <c r="L11" t="inlineStr">
@@ -2068,42 +2068,42 @@
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>DESPESA</t>
+          <t>TRANSMOVE GSL</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>1.4 DESPESA</t>
+          <t>1.4 TRANSMOVE GSL</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>1.4</t>
+          <t>1.4.4</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>TRANSMOVE GSL</t>
+          <t>BARUERI</t>
         </is>
       </c>
       <c r="H12" t="inlineStr">
         <is>
-          <t>1.4 TRANSMOVE GSL</t>
+          <t>1.4.4 BARUERI</t>
         </is>
       </c>
       <c r="I12" t="inlineStr">
         <is>
-          <t>1.4.4</t>
+          <t>1.4.4.2</t>
         </is>
       </c>
       <c r="J12" t="inlineStr">
         <is>
-          <t>BARUERI</t>
+          <t>ADMINISTRATIVO</t>
         </is>
       </c>
       <c r="K12" t="inlineStr">
         <is>
-          <t>1.4.4 BARUERI</t>
+          <t>1.4.4.2 ADMINISTRATIVO</t>
         </is>
       </c>
       <c r="L12" t="inlineStr">
@@ -2214,42 +2214,42 @@
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>DESPESA</t>
+          <t>TRANSMOVE GSL</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>1.4 DESPESA</t>
+          <t>1.4 TRANSMOVE GSL</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>1.4</t>
+          <t>1.4.1</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>TRANSMOVE GSL</t>
+          <t>PRESIDENTE PRUDENTE</t>
         </is>
       </c>
       <c r="H13" t="inlineStr">
         <is>
-          <t>1.4 TRANSMOVE GSL</t>
+          <t>1.4.1 PRESIDENTE PRUDENTE</t>
         </is>
       </c>
       <c r="I13" t="inlineStr">
         <is>
-          <t>1.4.1</t>
+          <t>1.4.1.2</t>
         </is>
       </c>
       <c r="J13" t="inlineStr">
         <is>
-          <t>PRESIDENTE PRUDENTE</t>
+          <t>ADMINISTRATIVO</t>
         </is>
       </c>
       <c r="K13" t="inlineStr">
         <is>
-          <t>1.4.1 PRESIDENTE PRUDENTE</t>
+          <t>1.4.1.2 ADMINISTRATIVO</t>
         </is>
       </c>
       <c r="L13" t="inlineStr">
@@ -2360,42 +2360,42 @@
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>DESPESA</t>
+          <t>TRANSMOVE GSL</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>1.4 DESPESA</t>
+          <t>1.4 TRANSMOVE GSL</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>1.4</t>
+          <t>1.4.1</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>TRANSMOVE GSL</t>
+          <t>PRESIDENTE PRUDENTE</t>
         </is>
       </c>
       <c r="H14" t="inlineStr">
         <is>
-          <t>1.4 TRANSMOVE GSL</t>
+          <t>1.4.1 PRESIDENTE PRUDENTE</t>
         </is>
       </c>
       <c r="I14" t="inlineStr">
         <is>
-          <t>1.4.1</t>
+          <t>1.4.1.1</t>
         </is>
       </c>
       <c r="J14" t="inlineStr">
         <is>
-          <t>PRESIDENTE PRUDENTE</t>
+          <t>TRANSPORTE</t>
         </is>
       </c>
       <c r="K14" t="inlineStr">
         <is>
-          <t>1.4.1 PRESIDENTE PRUDENTE</t>
+          <t>1.4.1.1 TRANSPORTE</t>
         </is>
       </c>
       <c r="L14" t="inlineStr">
@@ -2506,42 +2506,42 @@
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>DESPESA</t>
+          <t>TRANSMOVE GSL</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>1.4 DESPESA</t>
+          <t>1.4 TRANSMOVE GSL</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>1.4</t>
+          <t>1.4.1</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>TRANSMOVE GSL</t>
+          <t>PRESIDENTE PRUDENTE</t>
         </is>
       </c>
       <c r="H15" t="inlineStr">
         <is>
-          <t>1.4 TRANSMOVE GSL</t>
+          <t>1.4.1 PRESIDENTE PRUDENTE</t>
         </is>
       </c>
       <c r="I15" t="inlineStr">
         <is>
-          <t>1.4.1</t>
+          <t>1.4.1.1</t>
         </is>
       </c>
       <c r="J15" t="inlineStr">
         <is>
-          <t>PRESIDENTE PRUDENTE</t>
+          <t>TRANSPORTE</t>
         </is>
       </c>
       <c r="K15" t="inlineStr">
         <is>
-          <t>1.4.1 PRESIDENTE PRUDENTE</t>
+          <t>1.4.1.1 TRANSPORTE</t>
         </is>
       </c>
       <c r="L15" t="inlineStr">
@@ -2652,42 +2652,42 @@
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>DESPESA</t>
+          <t>TRANSMOVE GSL</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>1.4 DESPESA</t>
+          <t>1.4 TRANSMOVE GSL</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>1.4</t>
+          <t>1.4.1</t>
         </is>
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>TRANSMOVE GSL</t>
+          <t>PRESIDENTE PRUDENTE</t>
         </is>
       </c>
       <c r="H16" t="inlineStr">
         <is>
-          <t>1.4 TRANSMOVE GSL</t>
+          <t>1.4.1 PRESIDENTE PRUDENTE</t>
         </is>
       </c>
       <c r="I16" t="inlineStr">
         <is>
-          <t>1.4.1</t>
+          <t>1.4.1.1</t>
         </is>
       </c>
       <c r="J16" t="inlineStr">
         <is>
-          <t>PRESIDENTE PRUDENTE</t>
+          <t>TRANSPORTE</t>
         </is>
       </c>
       <c r="K16" t="inlineStr">
         <is>
-          <t>1.4.1 PRESIDENTE PRUDENTE</t>
+          <t>1.4.1.1 TRANSPORTE</t>
         </is>
       </c>
       <c r="L16" t="inlineStr">
@@ -2798,42 +2798,42 @@
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>DESPESA</t>
+          <t>TRANSMOVE GSL</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>1.4 DESPESA</t>
+          <t>1.4 TRANSMOVE GSL</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>1.4</t>
+          <t>1.4.3</t>
         </is>
       </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t>TRANSMOVE GSL</t>
+          <t>MARINGA</t>
         </is>
       </c>
       <c r="H17" t="inlineStr">
         <is>
-          <t>1.4 TRANSMOVE GSL</t>
+          <t>1.4.3 MARINGA</t>
         </is>
       </c>
       <c r="I17" t="inlineStr">
         <is>
-          <t>1.4.3</t>
+          <t>1.4.3.2</t>
         </is>
       </c>
       <c r="J17" t="inlineStr">
         <is>
-          <t>MARINGA</t>
+          <t>ADMINISTRATIVO</t>
         </is>
       </c>
       <c r="K17" t="inlineStr">
         <is>
-          <t>1.4.3 MARINGA</t>
+          <t>1.4.3.2 ADMINISTRATIVO</t>
         </is>
       </c>
       <c r="L17" t="inlineStr">
@@ -2944,42 +2944,42 @@
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>DESPESA</t>
+          <t>TRANSMOVE GSL</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>1.4 DESPESA</t>
+          <t>1.4 TRANSMOVE GSL</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>1.4</t>
+          <t>1.4.2</t>
         </is>
       </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t>TRANSMOVE GSL</t>
+          <t>DOURADOS</t>
         </is>
       </c>
       <c r="H18" t="inlineStr">
         <is>
-          <t>1.4 TRANSMOVE GSL</t>
+          <t>1.4.2 DOURADOS</t>
         </is>
       </c>
       <c r="I18" t="inlineStr">
         <is>
-          <t>1.4.2</t>
+          <t>1.4.2.2</t>
         </is>
       </c>
       <c r="J18" t="inlineStr">
         <is>
-          <t>DOURADOS</t>
+          <t>ADMINISTRATIVO</t>
         </is>
       </c>
       <c r="K18" t="inlineStr">
         <is>
-          <t>1.4.2 DOURADOS</t>
+          <t>1.4.2.2 ADMINISTRATIVO</t>
         </is>
       </c>
       <c r="L18" t="inlineStr">
@@ -3090,42 +3090,42 @@
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>DESPESA</t>
+          <t>TRANSMOVE GSL</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>1.4 DESPESA</t>
+          <t>1.4 TRANSMOVE GSL</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>1.4</t>
+          <t>1.4.1</t>
         </is>
       </c>
       <c r="G19" t="inlineStr">
         <is>
-          <t>TRANSMOVE GSL</t>
+          <t>PRESIDENTE PRUDENTE</t>
         </is>
       </c>
       <c r="H19" t="inlineStr">
         <is>
-          <t>1.4 TRANSMOVE GSL</t>
+          <t>1.4.1 PRESIDENTE PRUDENTE</t>
         </is>
       </c>
       <c r="I19" t="inlineStr">
         <is>
-          <t>1.4.1</t>
+          <t>1.4.1.2</t>
         </is>
       </c>
       <c r="J19" t="inlineStr">
         <is>
-          <t>PRESIDENTE PRUDENTE</t>
+          <t>ADMINISTRATIVO</t>
         </is>
       </c>
       <c r="K19" t="inlineStr">
         <is>
-          <t>1.4.1 PRESIDENTE PRUDENTE</t>
+          <t>1.4.1.2 ADMINISTRATIVO</t>
         </is>
       </c>
       <c r="L19" t="inlineStr">
@@ -3236,42 +3236,42 @@
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>DESPESA</t>
+          <t>TRANSMOVE GSL</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>1.4 DESPESA</t>
+          <t>1.4 TRANSMOVE GSL</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>1.4</t>
+          <t>1.4.1</t>
         </is>
       </c>
       <c r="G20" t="inlineStr">
         <is>
-          <t>TRANSMOVE GSL</t>
+          <t>PRESIDENTE PRUDENTE</t>
         </is>
       </c>
       <c r="H20" t="inlineStr">
         <is>
-          <t>1.4 TRANSMOVE GSL</t>
+          <t>1.4.1 PRESIDENTE PRUDENTE</t>
         </is>
       </c>
       <c r="I20" t="inlineStr">
         <is>
-          <t>1.4.1</t>
+          <t>1.4.1.2</t>
         </is>
       </c>
       <c r="J20" t="inlineStr">
         <is>
-          <t>PRESIDENTE PRUDENTE</t>
+          <t>ADMINISTRATIVO</t>
         </is>
       </c>
       <c r="K20" t="inlineStr">
         <is>
-          <t>1.4.1 PRESIDENTE PRUDENTE</t>
+          <t>1.4.1.2 ADMINISTRATIVO</t>
         </is>
       </c>
       <c r="L20" t="inlineStr">
@@ -3382,42 +3382,42 @@
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>DESPESA</t>
+          <t>TRANSMOVE GSL</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>1.4 DESPESA</t>
+          <t>1.4 TRANSMOVE GSL</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>1.4</t>
+          <t>1.4.1</t>
         </is>
       </c>
       <c r="G21" t="inlineStr">
         <is>
-          <t>TRANSMOVE GSL</t>
+          <t>PRESIDENTE PRUDENTE</t>
         </is>
       </c>
       <c r="H21" t="inlineStr">
         <is>
-          <t>1.4 TRANSMOVE GSL</t>
+          <t>1.4.1 PRESIDENTE PRUDENTE</t>
         </is>
       </c>
       <c r="I21" t="inlineStr">
         <is>
-          <t>1.4.1</t>
+          <t>1.4.1.2</t>
         </is>
       </c>
       <c r="J21" t="inlineStr">
         <is>
-          <t>PRESIDENTE PRUDENTE</t>
+          <t>ADMINISTRATIVO</t>
         </is>
       </c>
       <c r="K21" t="inlineStr">
         <is>
-          <t>1.4.1 PRESIDENTE PRUDENTE</t>
+          <t>1.4.1.2 ADMINISTRATIVO</t>
         </is>
       </c>
       <c r="L21" t="inlineStr">
@@ -3528,42 +3528,42 @@
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>DESPESA</t>
+          <t>TRANSMOVE GSL</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>1.4 DESPESA</t>
+          <t>1.4 TRANSMOVE GSL</t>
         </is>
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>1.4</t>
+          <t>1.4.1</t>
         </is>
       </c>
       <c r="G22" t="inlineStr">
         <is>
-          <t>TRANSMOVE GSL</t>
+          <t>PRESIDENTE PRUDENTE</t>
         </is>
       </c>
       <c r="H22" t="inlineStr">
         <is>
-          <t>1.4 TRANSMOVE GSL</t>
+          <t>1.4.1 PRESIDENTE PRUDENTE</t>
         </is>
       </c>
       <c r="I22" t="inlineStr">
         <is>
-          <t>1.4.1</t>
+          <t>1.4.1.1</t>
         </is>
       </c>
       <c r="J22" t="inlineStr">
         <is>
-          <t>PRESIDENTE PRUDENTE</t>
+          <t>TRANSPORTE</t>
         </is>
       </c>
       <c r="K22" t="inlineStr">
         <is>
-          <t>1.4.1 PRESIDENTE PRUDENTE</t>
+          <t>1.4.1.1 TRANSPORTE</t>
         </is>
       </c>
       <c r="L22" t="inlineStr">
@@ -3674,42 +3674,42 @@
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>DESPESA</t>
+          <t>TRANSMOVE GSL</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>1.4 DESPESA</t>
+          <t>1.4 TRANSMOVE GSL</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>1.4</t>
+          <t>1.4.1</t>
         </is>
       </c>
       <c r="G23" t="inlineStr">
         <is>
-          <t>TRANSMOVE GSL</t>
+          <t>PRESIDENTE PRUDENTE</t>
         </is>
       </c>
       <c r="H23" t="inlineStr">
         <is>
-          <t>1.4 TRANSMOVE GSL</t>
+          <t>1.4.1 PRESIDENTE PRUDENTE</t>
         </is>
       </c>
       <c r="I23" t="inlineStr">
         <is>
-          <t>1.4.1</t>
+          <t>1.4.1.1</t>
         </is>
       </c>
       <c r="J23" t="inlineStr">
         <is>
-          <t>PRESIDENTE PRUDENTE</t>
+          <t>TRANSPORTE</t>
         </is>
       </c>
       <c r="K23" t="inlineStr">
         <is>
-          <t>1.4.1 PRESIDENTE PRUDENTE</t>
+          <t>1.4.1.1 TRANSPORTE</t>
         </is>
       </c>
       <c r="L23" t="inlineStr">
@@ -3820,42 +3820,42 @@
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>DESPESA</t>
+          <t>TRANSMOVE GSL</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>1.4 DESPESA</t>
+          <t>1.4 TRANSMOVE GSL</t>
         </is>
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>1.4</t>
+          <t>1.4.1</t>
         </is>
       </c>
       <c r="G24" t="inlineStr">
         <is>
-          <t>TRANSMOVE GSL</t>
+          <t>PRESIDENTE PRUDENTE</t>
         </is>
       </c>
       <c r="H24" t="inlineStr">
         <is>
-          <t>1.4 TRANSMOVE GSL</t>
+          <t>1.4.1 PRESIDENTE PRUDENTE</t>
         </is>
       </c>
       <c r="I24" t="inlineStr">
         <is>
-          <t>1.4.1</t>
+          <t>1.4.1.1</t>
         </is>
       </c>
       <c r="J24" t="inlineStr">
         <is>
-          <t>PRESIDENTE PRUDENTE</t>
+          <t>TRANSPORTE</t>
         </is>
       </c>
       <c r="K24" t="inlineStr">
         <is>
-          <t>1.4.1 PRESIDENTE PRUDENTE</t>
+          <t>1.4.1.1 TRANSPORTE</t>
         </is>
       </c>
       <c r="L24" t="inlineStr">
@@ -3966,42 +3966,42 @@
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>DESPESA</t>
+          <t>TRANSMOVE GSL</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>1.4 DESPESA</t>
+          <t>1.4 TRANSMOVE GSL</t>
         </is>
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t>1.4</t>
+          <t>1.4.1</t>
         </is>
       </c>
       <c r="G25" t="inlineStr">
         <is>
-          <t>TRANSMOVE GSL</t>
+          <t>PRESIDENTE PRUDENTE</t>
         </is>
       </c>
       <c r="H25" t="inlineStr">
         <is>
-          <t>1.4 TRANSMOVE GSL</t>
+          <t>1.4.1 PRESIDENTE PRUDENTE</t>
         </is>
       </c>
       <c r="I25" t="inlineStr">
         <is>
-          <t>1.4.1</t>
+          <t>1.4.1.1</t>
         </is>
       </c>
       <c r="J25" t="inlineStr">
         <is>
-          <t>PRESIDENTE PRUDENTE</t>
+          <t>TRANSPORTE</t>
         </is>
       </c>
       <c r="K25" t="inlineStr">
         <is>
-          <t>1.4.1 PRESIDENTE PRUDENTE</t>
+          <t>1.4.1.1 TRANSPORTE</t>
         </is>
       </c>
       <c r="L25" t="inlineStr">
@@ -4112,42 +4112,42 @@
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>DESPESA</t>
+          <t>TRANSMOVE GSL</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>1.4 DESPESA</t>
+          <t>1.4 TRANSMOVE GSL</t>
         </is>
       </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t>1.4</t>
+          <t>1.4.1</t>
         </is>
       </c>
       <c r="G26" t="inlineStr">
         <is>
-          <t>TRANSMOVE GSL</t>
+          <t>PRESIDENTE PRUDENTE</t>
         </is>
       </c>
       <c r="H26" t="inlineStr">
         <is>
-          <t>1.4 TRANSMOVE GSL</t>
+          <t>1.4.1 PRESIDENTE PRUDENTE</t>
         </is>
       </c>
       <c r="I26" t="inlineStr">
         <is>
-          <t>1.4.1</t>
+          <t>1.4.1.1</t>
         </is>
       </c>
       <c r="J26" t="inlineStr">
         <is>
-          <t>PRESIDENTE PRUDENTE</t>
+          <t>TRANSPORTE</t>
         </is>
       </c>
       <c r="K26" t="inlineStr">
         <is>
-          <t>1.4.1 PRESIDENTE PRUDENTE</t>
+          <t>1.4.1.1 TRANSPORTE</t>
         </is>
       </c>
       <c r="L26" t="inlineStr">
@@ -4258,42 +4258,42 @@
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>DESPESA</t>
+          <t>TRANSMOVE GSL</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>1.4 DESPESA</t>
+          <t>1.4 TRANSMOVE GSL</t>
         </is>
       </c>
       <c r="F27" t="inlineStr">
         <is>
-          <t>1.4</t>
+          <t>1.4.1</t>
         </is>
       </c>
       <c r="G27" t="inlineStr">
         <is>
-          <t>TRANSMOVE GSL</t>
+          <t>PRESIDENTE PRUDENTE</t>
         </is>
       </c>
       <c r="H27" t="inlineStr">
         <is>
-          <t>1.4 TRANSMOVE GSL</t>
+          <t>1.4.1 PRESIDENTE PRUDENTE</t>
         </is>
       </c>
       <c r="I27" t="inlineStr">
         <is>
-          <t>1.4.1</t>
+          <t>1.4.1.1</t>
         </is>
       </c>
       <c r="J27" t="inlineStr">
         <is>
-          <t>PRESIDENTE PRUDENTE</t>
+          <t>TRANSPORTE</t>
         </is>
       </c>
       <c r="K27" t="inlineStr">
         <is>
-          <t>1.4.1 PRESIDENTE PRUDENTE</t>
+          <t>1.4.1.1 TRANSPORTE</t>
         </is>
       </c>
       <c r="L27" t="inlineStr">
@@ -4404,42 +4404,42 @@
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>DESPESA</t>
+          <t>TRANSMOVE GSL</t>
         </is>
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>1.4 DESPESA</t>
+          <t>1.4 TRANSMOVE GSL</t>
         </is>
       </c>
       <c r="F28" t="inlineStr">
         <is>
-          <t>1.4</t>
+          <t>1.4.1</t>
         </is>
       </c>
       <c r="G28" t="inlineStr">
         <is>
-          <t>TRANSMOVE GSL</t>
+          <t>PRESIDENTE PRUDENTE</t>
         </is>
       </c>
       <c r="H28" t="inlineStr">
         <is>
-          <t>1.4 TRANSMOVE GSL</t>
+          <t>1.4.1 PRESIDENTE PRUDENTE</t>
         </is>
       </c>
       <c r="I28" t="inlineStr">
         <is>
-          <t>1.4.1</t>
+          <t>1.4.1.1</t>
         </is>
       </c>
       <c r="J28" t="inlineStr">
         <is>
-          <t>PRESIDENTE PRUDENTE</t>
+          <t>TRANSPORTE</t>
         </is>
       </c>
       <c r="K28" t="inlineStr">
         <is>
-          <t>1.4.1 PRESIDENTE PRUDENTE</t>
+          <t>1.4.1.1 TRANSPORTE</t>
         </is>
       </c>
       <c r="L28" t="inlineStr">
@@ -4550,42 +4550,42 @@
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>DESPESA</t>
+          <t>TRANSMOVE GSL</t>
         </is>
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>1.4 DESPESA</t>
+          <t>1.4 TRANSMOVE GSL</t>
         </is>
       </c>
       <c r="F29" t="inlineStr">
         <is>
-          <t>1.4</t>
+          <t>1.4.1</t>
         </is>
       </c>
       <c r="G29" t="inlineStr">
         <is>
-          <t>TRANSMOVE GSL</t>
+          <t>PRESIDENTE PRUDENTE</t>
         </is>
       </c>
       <c r="H29" t="inlineStr">
         <is>
-          <t>1.4 TRANSMOVE GSL</t>
+          <t>1.4.1 PRESIDENTE PRUDENTE</t>
         </is>
       </c>
       <c r="I29" t="inlineStr">
         <is>
-          <t>1.4.1</t>
+          <t>1.4.1.1</t>
         </is>
       </c>
       <c r="J29" t="inlineStr">
         <is>
-          <t>PRESIDENTE PRUDENTE</t>
+          <t>TRANSPORTE</t>
         </is>
       </c>
       <c r="K29" t="inlineStr">
         <is>
-          <t>1.4.1 PRESIDENTE PRUDENTE</t>
+          <t>1.4.1.1 TRANSPORTE</t>
         </is>
       </c>
       <c r="L29" t="inlineStr">
@@ -4696,42 +4696,42 @@
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>DESPESA</t>
+          <t>TRANSMOVE GSL</t>
         </is>
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>1.4 DESPESA</t>
+          <t>1.4 TRANSMOVE GSL</t>
         </is>
       </c>
       <c r="F30" t="inlineStr">
         <is>
-          <t>1.4</t>
+          <t>1.4.1</t>
         </is>
       </c>
       <c r="G30" t="inlineStr">
         <is>
-          <t>TRANSMOVE GSL</t>
+          <t>PRESIDENTE PRUDENTE</t>
         </is>
       </c>
       <c r="H30" t="inlineStr">
         <is>
-          <t>1.4 TRANSMOVE GSL</t>
+          <t>1.4.1 PRESIDENTE PRUDENTE</t>
         </is>
       </c>
       <c r="I30" t="inlineStr">
         <is>
-          <t>1.4.1</t>
+          <t>1.4.1.1</t>
         </is>
       </c>
       <c r="J30" t="inlineStr">
         <is>
-          <t>PRESIDENTE PRUDENTE</t>
+          <t>TRANSPORTE</t>
         </is>
       </c>
       <c r="K30" t="inlineStr">
         <is>
-          <t>1.4.1 PRESIDENTE PRUDENTE</t>
+          <t>1.4.1.1 TRANSPORTE</t>
         </is>
       </c>
       <c r="L30" t="inlineStr">
@@ -4842,42 +4842,42 @@
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>DESPESA</t>
+          <t>TRANSMOVE GSL</t>
         </is>
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>1.4 DESPESA</t>
+          <t>1.4 TRANSMOVE GSL</t>
         </is>
       </c>
       <c r="F31" t="inlineStr">
         <is>
-          <t>1.4</t>
+          <t>1.4.1</t>
         </is>
       </c>
       <c r="G31" t="inlineStr">
         <is>
-          <t>TRANSMOVE GSL</t>
+          <t>PRESIDENTE PRUDENTE</t>
         </is>
       </c>
       <c r="H31" t="inlineStr">
         <is>
-          <t>1.4 TRANSMOVE GSL</t>
+          <t>1.4.1 PRESIDENTE PRUDENTE</t>
         </is>
       </c>
       <c r="I31" t="inlineStr">
         <is>
-          <t>1.4.1</t>
+          <t>1.4.1.1</t>
         </is>
       </c>
       <c r="J31" t="inlineStr">
         <is>
-          <t>PRESIDENTE PRUDENTE</t>
+          <t>TRANSPORTE</t>
         </is>
       </c>
       <c r="K31" t="inlineStr">
         <is>
-          <t>1.4.1 PRESIDENTE PRUDENTE</t>
+          <t>1.4.1.1 TRANSPORTE</t>
         </is>
       </c>
       <c r="L31" t="inlineStr">
@@ -4988,42 +4988,42 @@
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>DESPESA</t>
+          <t>TRANSMOVE GSL</t>
         </is>
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>1.4 DESPESA</t>
+          <t>1.4 TRANSMOVE GSL</t>
         </is>
       </c>
       <c r="F32" t="inlineStr">
         <is>
-          <t>1.4</t>
+          <t>1.4.1</t>
         </is>
       </c>
       <c r="G32" t="inlineStr">
         <is>
-          <t>TRANSMOVE GSL</t>
+          <t>PRESIDENTE PRUDENTE</t>
         </is>
       </c>
       <c r="H32" t="inlineStr">
         <is>
-          <t>1.4 TRANSMOVE GSL</t>
+          <t>1.4.1 PRESIDENTE PRUDENTE</t>
         </is>
       </c>
       <c r="I32" t="inlineStr">
         <is>
-          <t>1.4.1</t>
+          <t>1.4.1.1</t>
         </is>
       </c>
       <c r="J32" t="inlineStr">
         <is>
-          <t>PRESIDENTE PRUDENTE</t>
+          <t>TRANSPORTE</t>
         </is>
       </c>
       <c r="K32" t="inlineStr">
         <is>
-          <t>1.4.1 PRESIDENTE PRUDENTE</t>
+          <t>1.4.1.1 TRANSPORTE</t>
         </is>
       </c>
       <c r="L32" t="inlineStr">
@@ -5134,42 +5134,42 @@
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>DESPESA</t>
+          <t>TRANSMOVE GSL</t>
         </is>
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>1.4 DESPESA</t>
+          <t>1.4 TRANSMOVE GSL</t>
         </is>
       </c>
       <c r="F33" t="inlineStr">
         <is>
-          <t>1.4</t>
+          <t>1.4.1</t>
         </is>
       </c>
       <c r="G33" t="inlineStr">
         <is>
-          <t>TRANSMOVE GSL</t>
+          <t>PRESIDENTE PRUDENTE</t>
         </is>
       </c>
       <c r="H33" t="inlineStr">
         <is>
-          <t>1.4 TRANSMOVE GSL</t>
+          <t>1.4.1 PRESIDENTE PRUDENTE</t>
         </is>
       </c>
       <c r="I33" t="inlineStr">
         <is>
-          <t>1.4.1</t>
+          <t>1.4.1.2</t>
         </is>
       </c>
       <c r="J33" t="inlineStr">
         <is>
-          <t>PRESIDENTE PRUDENTE</t>
+          <t>ADMINISTRATIVO</t>
         </is>
       </c>
       <c r="K33" t="inlineStr">
         <is>
-          <t>1.4.1 PRESIDENTE PRUDENTE</t>
+          <t>1.4.1.2 ADMINISTRATIVO</t>
         </is>
       </c>
       <c r="L33" t="inlineStr">
@@ -5280,42 +5280,42 @@
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>DESPESA</t>
+          <t>TRANSMOVE GSL</t>
         </is>
       </c>
       <c r="E34" t="inlineStr">
         <is>
-          <t>1.4 DESPESA</t>
+          <t>1.4 TRANSMOVE GSL</t>
         </is>
       </c>
       <c r="F34" t="inlineStr">
         <is>
-          <t>1.4</t>
+          <t>1.4.1</t>
         </is>
       </c>
       <c r="G34" t="inlineStr">
         <is>
-          <t>TRANSMOVE GSL</t>
+          <t>PRESIDENTE PRUDENTE</t>
         </is>
       </c>
       <c r="H34" t="inlineStr">
         <is>
-          <t>1.4 TRANSMOVE GSL</t>
+          <t>1.4.1 PRESIDENTE PRUDENTE</t>
         </is>
       </c>
       <c r="I34" t="inlineStr">
         <is>
-          <t>1.4.1</t>
+          <t>1.4.1.1</t>
         </is>
       </c>
       <c r="J34" t="inlineStr">
         <is>
-          <t>PRESIDENTE PRUDENTE</t>
+          <t>TRANSPORTE</t>
         </is>
       </c>
       <c r="K34" t="inlineStr">
         <is>
-          <t>1.4.1 PRESIDENTE PRUDENTE</t>
+          <t>1.4.1.1 TRANSPORTE</t>
         </is>
       </c>
       <c r="L34" t="inlineStr">
@@ -5426,42 +5426,42 @@
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>DESPESA</t>
+          <t>TRANSMOVE GSL</t>
         </is>
       </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t>1.4 DESPESA</t>
+          <t>1.4 TRANSMOVE GSL</t>
         </is>
       </c>
       <c r="F35" t="inlineStr">
         <is>
-          <t>1.4</t>
+          <t>1.4.1</t>
         </is>
       </c>
       <c r="G35" t="inlineStr">
         <is>
-          <t>TRANSMOVE GSL</t>
+          <t>PRESIDENTE PRUDENTE</t>
         </is>
       </c>
       <c r="H35" t="inlineStr">
         <is>
-          <t>1.4 TRANSMOVE GSL</t>
+          <t>1.4.1 PRESIDENTE PRUDENTE</t>
         </is>
       </c>
       <c r="I35" t="inlineStr">
         <is>
-          <t>1.4.1</t>
+          <t>1.4.1.1</t>
         </is>
       </c>
       <c r="J35" t="inlineStr">
         <is>
-          <t>PRESIDENTE PRUDENTE</t>
+          <t>TRANSPORTE</t>
         </is>
       </c>
       <c r="K35" t="inlineStr">
         <is>
-          <t>1.4.1 PRESIDENTE PRUDENTE</t>
+          <t>1.4.1.1 TRANSPORTE</t>
         </is>
       </c>
       <c r="L35" t="inlineStr">
@@ -5572,42 +5572,42 @@
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>DESPESA</t>
+          <t>TRANSMOVE GSL</t>
         </is>
       </c>
       <c r="E36" t="inlineStr">
         <is>
-          <t>1.4 DESPESA</t>
+          <t>1.4 TRANSMOVE GSL</t>
         </is>
       </c>
       <c r="F36" t="inlineStr">
         <is>
-          <t>1.4</t>
+          <t>1.4.1</t>
         </is>
       </c>
       <c r="G36" t="inlineStr">
         <is>
-          <t>TRANSMOVE GSL</t>
+          <t>PRESIDENTE PRUDENTE</t>
         </is>
       </c>
       <c r="H36" t="inlineStr">
         <is>
-          <t>1.4 TRANSMOVE GSL</t>
+          <t>1.4.1 PRESIDENTE PRUDENTE</t>
         </is>
       </c>
       <c r="I36" t="inlineStr">
         <is>
-          <t>1.4.1</t>
+          <t>1.4.1.1</t>
         </is>
       </c>
       <c r="J36" t="inlineStr">
         <is>
-          <t>PRESIDENTE PRUDENTE</t>
+          <t>TRANSPORTE</t>
         </is>
       </c>
       <c r="K36" t="inlineStr">
         <is>
-          <t>1.4.1 PRESIDENTE PRUDENTE</t>
+          <t>1.4.1.1 TRANSPORTE</t>
         </is>
       </c>
       <c r="L36" t="inlineStr">
@@ -5718,42 +5718,42 @@
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>DESPESA</t>
+          <t>TRANSMOVE GSL</t>
         </is>
       </c>
       <c r="E37" t="inlineStr">
         <is>
-          <t>1.4 DESPESA</t>
+          <t>1.4 TRANSMOVE GSL</t>
         </is>
       </c>
       <c r="F37" t="inlineStr">
         <is>
-          <t>1.4</t>
+          <t>1.4.1</t>
         </is>
       </c>
       <c r="G37" t="inlineStr">
         <is>
-          <t>TRANSMOVE GSL</t>
+          <t>PRESIDENTE PRUDENTE</t>
         </is>
       </c>
       <c r="H37" t="inlineStr">
         <is>
-          <t>1.4 TRANSMOVE GSL</t>
+          <t>1.4.1 PRESIDENTE PRUDENTE</t>
         </is>
       </c>
       <c r="I37" t="inlineStr">
         <is>
-          <t>1.4.1</t>
+          <t>1.4.1.1</t>
         </is>
       </c>
       <c r="J37" t="inlineStr">
         <is>
-          <t>PRESIDENTE PRUDENTE</t>
+          <t>TRANSPORTE</t>
         </is>
       </c>
       <c r="K37" t="inlineStr">
         <is>
-          <t>1.4.1 PRESIDENTE PRUDENTE</t>
+          <t>1.4.1.1 TRANSPORTE</t>
         </is>
       </c>
       <c r="L37" t="inlineStr">
@@ -5864,42 +5864,42 @@
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>DESPESA</t>
+          <t>TRANSMOVE GSL</t>
         </is>
       </c>
       <c r="E38" t="inlineStr">
         <is>
-          <t>1.4 DESPESA</t>
+          <t>1.4 TRANSMOVE GSL</t>
         </is>
       </c>
       <c r="F38" t="inlineStr">
         <is>
-          <t>1.4</t>
+          <t>1.4.1</t>
         </is>
       </c>
       <c r="G38" t="inlineStr">
         <is>
-          <t>TRANSMOVE GSL</t>
+          <t>PRESIDENTE PRUDENTE</t>
         </is>
       </c>
       <c r="H38" t="inlineStr">
         <is>
-          <t>1.4 TRANSMOVE GSL</t>
+          <t>1.4.1 PRESIDENTE PRUDENTE</t>
         </is>
       </c>
       <c r="I38" t="inlineStr">
         <is>
-          <t>1.4.1</t>
+          <t>1.4.1.1</t>
         </is>
       </c>
       <c r="J38" t="inlineStr">
         <is>
-          <t>PRESIDENTE PRUDENTE</t>
+          <t>TRANSPORTE</t>
         </is>
       </c>
       <c r="K38" t="inlineStr">
         <is>
-          <t>1.4.1 PRESIDENTE PRUDENTE</t>
+          <t>1.4.1.1 TRANSPORTE</t>
         </is>
       </c>
       <c r="L38" t="inlineStr">
@@ -6010,42 +6010,42 @@
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>DESPESA</t>
+          <t>TRANSMOVE GSL</t>
         </is>
       </c>
       <c r="E39" t="inlineStr">
         <is>
-          <t>1.4 DESPESA</t>
+          <t>1.4 TRANSMOVE GSL</t>
         </is>
       </c>
       <c r="F39" t="inlineStr">
         <is>
-          <t>1.4</t>
+          <t>1.4.1</t>
         </is>
       </c>
       <c r="G39" t="inlineStr">
         <is>
-          <t>TRANSMOVE GSL</t>
+          <t>PRESIDENTE PRUDENTE</t>
         </is>
       </c>
       <c r="H39" t="inlineStr">
         <is>
-          <t>1.4 TRANSMOVE GSL</t>
+          <t>1.4.1 PRESIDENTE PRUDENTE</t>
         </is>
       </c>
       <c r="I39" t="inlineStr">
         <is>
-          <t>1.4.1</t>
+          <t>1.4.1.1</t>
         </is>
       </c>
       <c r="J39" t="inlineStr">
         <is>
-          <t>PRESIDENTE PRUDENTE</t>
+          <t>TRANSPORTE</t>
         </is>
       </c>
       <c r="K39" t="inlineStr">
         <is>
-          <t>1.4.1 PRESIDENTE PRUDENTE</t>
+          <t>1.4.1.1 TRANSPORTE</t>
         </is>
       </c>
       <c r="L39" t="inlineStr">
@@ -6156,42 +6156,42 @@
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>DESPESA</t>
+          <t>TRANSMOVE GSL</t>
         </is>
       </c>
       <c r="E40" t="inlineStr">
         <is>
-          <t>1.4 DESPESA</t>
+          <t>1.4 TRANSMOVE GSL</t>
         </is>
       </c>
       <c r="F40" t="inlineStr">
         <is>
-          <t>1.4</t>
+          <t>1.4.4</t>
         </is>
       </c>
       <c r="G40" t="inlineStr">
         <is>
-          <t>TRANSMOVE GSL</t>
+          <t>BARUERI</t>
         </is>
       </c>
       <c r="H40" t="inlineStr">
         <is>
-          <t>1.4 TRANSMOVE GSL</t>
+          <t>1.4.4 BARUERI</t>
         </is>
       </c>
       <c r="I40" t="inlineStr">
         <is>
-          <t>1.4.4</t>
+          <t>1.4.4.2</t>
         </is>
       </c>
       <c r="J40" t="inlineStr">
         <is>
-          <t>BARUERI</t>
+          <t>ADMINISTRATIVO</t>
         </is>
       </c>
       <c r="K40" t="inlineStr">
         <is>
-          <t>1.4.4 BARUERI</t>
+          <t>1.4.4.2 ADMINISTRATIVO</t>
         </is>
       </c>
       <c r="L40" t="inlineStr">
@@ -6302,42 +6302,42 @@
       </c>
       <c r="D41" t="inlineStr">
         <is>
-          <t>DESPESA</t>
+          <t>TRANSMOVE GSL</t>
         </is>
       </c>
       <c r="E41" t="inlineStr">
         <is>
-          <t>1.4 DESPESA</t>
+          <t>1.4 TRANSMOVE GSL</t>
         </is>
       </c>
       <c r="F41" t="inlineStr">
         <is>
-          <t>1.4</t>
+          <t>1.4.1</t>
         </is>
       </c>
       <c r="G41" t="inlineStr">
         <is>
-          <t>TRANSMOVE GSL</t>
+          <t>PRESIDENTE PRUDENTE</t>
         </is>
       </c>
       <c r="H41" t="inlineStr">
         <is>
-          <t>1.4 TRANSMOVE GSL</t>
+          <t>1.4.1 PRESIDENTE PRUDENTE</t>
         </is>
       </c>
       <c r="I41" t="inlineStr">
         <is>
-          <t>1.4.1</t>
+          <t>1.4.1.1</t>
         </is>
       </c>
       <c r="J41" t="inlineStr">
         <is>
-          <t>PRESIDENTE PRUDENTE</t>
+          <t>TRANSPORTE</t>
         </is>
       </c>
       <c r="K41" t="inlineStr">
         <is>
-          <t>1.4.1 PRESIDENTE PRUDENTE</t>
+          <t>1.4.1.1 TRANSPORTE</t>
         </is>
       </c>
       <c r="L41" t="inlineStr">
@@ -6448,42 +6448,42 @@
       </c>
       <c r="D42" t="inlineStr">
         <is>
-          <t>DESPESA</t>
+          <t>TRANSMOVE GSL</t>
         </is>
       </c>
       <c r="E42" t="inlineStr">
         <is>
-          <t>1.4 DESPESA</t>
+          <t>1.4 TRANSMOVE GSL</t>
         </is>
       </c>
       <c r="F42" t="inlineStr">
         <is>
-          <t>1.4</t>
+          <t>1.4.1</t>
         </is>
       </c>
       <c r="G42" t="inlineStr">
         <is>
-          <t>TRANSMOVE GSL</t>
+          <t>PRESIDENTE PRUDENTE</t>
         </is>
       </c>
       <c r="H42" t="inlineStr">
         <is>
-          <t>1.4 TRANSMOVE GSL</t>
+          <t>1.4.1 PRESIDENTE PRUDENTE</t>
         </is>
       </c>
       <c r="I42" t="inlineStr">
         <is>
-          <t>1.4.1</t>
+          <t>1.4.1.1</t>
         </is>
       </c>
       <c r="J42" t="inlineStr">
         <is>
-          <t>PRESIDENTE PRUDENTE</t>
+          <t>TRANSPORTE</t>
         </is>
       </c>
       <c r="K42" t="inlineStr">
         <is>
-          <t>1.4.1 PRESIDENTE PRUDENTE</t>
+          <t>1.4.1.1 TRANSPORTE</t>
         </is>
       </c>
       <c r="L42" t="inlineStr">
@@ -6594,42 +6594,42 @@
       </c>
       <c r="D43" t="inlineStr">
         <is>
-          <t>DESPESA</t>
+          <t>TRANSMOVE GSL</t>
         </is>
       </c>
       <c r="E43" t="inlineStr">
         <is>
-          <t>1.4 DESPESA</t>
+          <t>1.4 TRANSMOVE GSL</t>
         </is>
       </c>
       <c r="F43" t="inlineStr">
         <is>
-          <t>1.4</t>
+          <t>1.4.1</t>
         </is>
       </c>
       <c r="G43" t="inlineStr">
         <is>
-          <t>TRANSMOVE GSL</t>
+          <t>PRESIDENTE PRUDENTE</t>
         </is>
       </c>
       <c r="H43" t="inlineStr">
         <is>
-          <t>1.4 TRANSMOVE GSL</t>
+          <t>1.4.1 PRESIDENTE PRUDENTE</t>
         </is>
       </c>
       <c r="I43" t="inlineStr">
         <is>
-          <t>1.4.1</t>
+          <t>1.4.1.1</t>
         </is>
       </c>
       <c r="J43" t="inlineStr">
         <is>
-          <t>PRESIDENTE PRUDENTE</t>
+          <t>TRANSPORTE</t>
         </is>
       </c>
       <c r="K43" t="inlineStr">
         <is>
-          <t>1.4.1 PRESIDENTE PRUDENTE</t>
+          <t>1.4.1.1 TRANSPORTE</t>
         </is>
       </c>
       <c r="L43" t="inlineStr">
@@ -6740,42 +6740,42 @@
       </c>
       <c r="D44" t="inlineStr">
         <is>
-          <t>DESPESA</t>
+          <t>TRANSMOVE GSL</t>
         </is>
       </c>
       <c r="E44" t="inlineStr">
         <is>
-          <t>1.4 DESPESA</t>
+          <t>1.4 TRANSMOVE GSL</t>
         </is>
       </c>
       <c r="F44" t="inlineStr">
         <is>
-          <t>1.4</t>
+          <t>1.4.1</t>
         </is>
       </c>
       <c r="G44" t="inlineStr">
         <is>
-          <t>TRANSMOVE GSL</t>
+          <t>PRESIDENTE PRUDENTE</t>
         </is>
       </c>
       <c r="H44" t="inlineStr">
         <is>
-          <t>1.4 TRANSMOVE GSL</t>
+          <t>1.4.1 PRESIDENTE PRUDENTE</t>
         </is>
       </c>
       <c r="I44" t="inlineStr">
         <is>
-          <t>1.4.1</t>
+          <t>1.4.1.1</t>
         </is>
       </c>
       <c r="J44" t="inlineStr">
         <is>
-          <t>PRESIDENTE PRUDENTE</t>
+          <t>TRANSPORTE</t>
         </is>
       </c>
       <c r="K44" t="inlineStr">
         <is>
-          <t>1.4.1 PRESIDENTE PRUDENTE</t>
+          <t>1.4.1.1 TRANSPORTE</t>
         </is>
       </c>
       <c r="L44" t="inlineStr">
@@ -6886,42 +6886,42 @@
       </c>
       <c r="D45" t="inlineStr">
         <is>
-          <t>DESPESA</t>
+          <t>TRANSMOVE GSL</t>
         </is>
       </c>
       <c r="E45" t="inlineStr">
         <is>
-          <t>1.4 DESPESA</t>
+          <t>1.4 TRANSMOVE GSL</t>
         </is>
       </c>
       <c r="F45" t="inlineStr">
         <is>
-          <t>1.4</t>
+          <t>1.4.1</t>
         </is>
       </c>
       <c r="G45" t="inlineStr">
         <is>
-          <t>TRANSMOVE GSL</t>
+          <t>PRESIDENTE PRUDENTE</t>
         </is>
       </c>
       <c r="H45" t="inlineStr">
         <is>
-          <t>1.4 TRANSMOVE GSL</t>
+          <t>1.4.1 PRESIDENTE PRUDENTE</t>
         </is>
       </c>
       <c r="I45" t="inlineStr">
         <is>
-          <t>1.4.1</t>
+          <t>1.4.1.1</t>
         </is>
       </c>
       <c r="J45" t="inlineStr">
         <is>
-          <t>PRESIDENTE PRUDENTE</t>
+          <t>TRANSPORTE</t>
         </is>
       </c>
       <c r="K45" t="inlineStr">
         <is>
-          <t>1.4.1 PRESIDENTE PRUDENTE</t>
+          <t>1.4.1.1 TRANSPORTE</t>
         </is>
       </c>
       <c r="L45" t="inlineStr">
@@ -7032,42 +7032,42 @@
       </c>
       <c r="D46" t="inlineStr">
         <is>
-          <t>DESPESA</t>
+          <t>TRANSMOVE GSL</t>
         </is>
       </c>
       <c r="E46" t="inlineStr">
         <is>
-          <t>1.4 DESPESA</t>
+          <t>1.4 TRANSMOVE GSL</t>
         </is>
       </c>
       <c r="F46" t="inlineStr">
         <is>
-          <t>1.4</t>
+          <t>1.4.1</t>
         </is>
       </c>
       <c r="G46" t="inlineStr">
         <is>
-          <t>TRANSMOVE GSL</t>
+          <t>PRESIDENTE PRUDENTE</t>
         </is>
       </c>
       <c r="H46" t="inlineStr">
         <is>
-          <t>1.4 TRANSMOVE GSL</t>
+          <t>1.4.1 PRESIDENTE PRUDENTE</t>
         </is>
       </c>
       <c r="I46" t="inlineStr">
         <is>
-          <t>1.4.1</t>
+          <t>1.4.1.1</t>
         </is>
       </c>
       <c r="J46" t="inlineStr">
         <is>
-          <t>PRESIDENTE PRUDENTE</t>
+          <t>TRANSPORTE</t>
         </is>
       </c>
       <c r="K46" t="inlineStr">
         <is>
-          <t>1.4.1 PRESIDENTE PRUDENTE</t>
+          <t>1.4.1.1 TRANSPORTE</t>
         </is>
       </c>
       <c r="L46" t="inlineStr">
@@ -7178,42 +7178,42 @@
       </c>
       <c r="D47" t="inlineStr">
         <is>
-          <t>DESPESA</t>
+          <t>TRANSMOVE GSL</t>
         </is>
       </c>
       <c r="E47" t="inlineStr">
         <is>
-          <t>1.4 DESPESA</t>
+          <t>1.4 TRANSMOVE GSL</t>
         </is>
       </c>
       <c r="F47" t="inlineStr">
         <is>
-          <t>1.4</t>
+          <t>1.4.1</t>
         </is>
       </c>
       <c r="G47" t="inlineStr">
         <is>
-          <t>TRANSMOVE GSL</t>
+          <t>PRESIDENTE PRUDENTE</t>
         </is>
       </c>
       <c r="H47" t="inlineStr">
         <is>
-          <t>1.4 TRANSMOVE GSL</t>
+          <t>1.4.1 PRESIDENTE PRUDENTE</t>
         </is>
       </c>
       <c r="I47" t="inlineStr">
         <is>
-          <t>1.4.1</t>
+          <t>1.4.1.2</t>
         </is>
       </c>
       <c r="J47" t="inlineStr">
         <is>
-          <t>PRESIDENTE PRUDENTE</t>
+          <t>ADMINISTRATIVO</t>
         </is>
       </c>
       <c r="K47" t="inlineStr">
         <is>
-          <t>1.4.1 PRESIDENTE PRUDENTE</t>
+          <t>1.4.1.2 ADMINISTRATIVO</t>
         </is>
       </c>
       <c r="L47" t="inlineStr">
@@ -7324,42 +7324,42 @@
       </c>
       <c r="D48" t="inlineStr">
         <is>
-          <t>DESPESA</t>
+          <t>TRANSMOVE GSL</t>
         </is>
       </c>
       <c r="E48" t="inlineStr">
         <is>
-          <t>1.4 DESPESA</t>
+          <t>1.4 TRANSMOVE GSL</t>
         </is>
       </c>
       <c r="F48" t="inlineStr">
         <is>
-          <t>1.4</t>
+          <t>1.4.1</t>
         </is>
       </c>
       <c r="G48" t="inlineStr">
         <is>
-          <t>TRANSMOVE GSL</t>
+          <t>PRESIDENTE PRUDENTE</t>
         </is>
       </c>
       <c r="H48" t="inlineStr">
         <is>
-          <t>1.4 TRANSMOVE GSL</t>
+          <t>1.4.1 PRESIDENTE PRUDENTE</t>
         </is>
       </c>
       <c r="I48" t="inlineStr">
         <is>
-          <t>1.4.1</t>
+          <t>1.4.1.1</t>
         </is>
       </c>
       <c r="J48" t="inlineStr">
         <is>
-          <t>PRESIDENTE PRUDENTE</t>
+          <t>TRANSPORTE</t>
         </is>
       </c>
       <c r="K48" t="inlineStr">
         <is>
-          <t>1.4.1 PRESIDENTE PRUDENTE</t>
+          <t>1.4.1.1 TRANSPORTE</t>
         </is>
       </c>
       <c r="L48" t="inlineStr">
@@ -7470,42 +7470,42 @@
       </c>
       <c r="D49" t="inlineStr">
         <is>
-          <t>DESPESA</t>
+          <t>TRANSMOVE GSL</t>
         </is>
       </c>
       <c r="E49" t="inlineStr">
         <is>
-          <t>1.4 DESPESA</t>
+          <t>1.4 TRANSMOVE GSL</t>
         </is>
       </c>
       <c r="F49" t="inlineStr">
         <is>
-          <t>1.4</t>
+          <t>1.4.1</t>
         </is>
       </c>
       <c r="G49" t="inlineStr">
         <is>
-          <t>TRANSMOVE GSL</t>
+          <t>PRESIDENTE PRUDENTE</t>
         </is>
       </c>
       <c r="H49" t="inlineStr">
         <is>
-          <t>1.4 TRANSMOVE GSL</t>
+          <t>1.4.1 PRESIDENTE PRUDENTE</t>
         </is>
       </c>
       <c r="I49" t="inlineStr">
         <is>
-          <t>1.4.1</t>
+          <t>1.4.1.1</t>
         </is>
       </c>
       <c r="J49" t="inlineStr">
         <is>
-          <t>PRESIDENTE PRUDENTE</t>
+          <t>TRANSPORTE</t>
         </is>
       </c>
       <c r="K49" t="inlineStr">
         <is>
-          <t>1.4.1 PRESIDENTE PRUDENTE</t>
+          <t>1.4.1.1 TRANSPORTE</t>
         </is>
       </c>
       <c r="L49" t="inlineStr">
@@ -7616,42 +7616,42 @@
       </c>
       <c r="D50" t="inlineStr">
         <is>
-          <t>DESPESA</t>
+          <t>TRANSMOVE GSL</t>
         </is>
       </c>
       <c r="E50" t="inlineStr">
         <is>
-          <t>1.4 DESPESA</t>
+          <t>1.4 TRANSMOVE GSL</t>
         </is>
       </c>
       <c r="F50" t="inlineStr">
         <is>
-          <t>1.4</t>
+          <t>1.4.1</t>
         </is>
       </c>
       <c r="G50" t="inlineStr">
         <is>
-          <t>TRANSMOVE GSL</t>
+          <t>PRESIDENTE PRUDENTE</t>
         </is>
       </c>
       <c r="H50" t="inlineStr">
         <is>
-          <t>1.4 TRANSMOVE GSL</t>
+          <t>1.4.1 PRESIDENTE PRUDENTE</t>
         </is>
       </c>
       <c r="I50" t="inlineStr">
         <is>
-          <t>1.4.1</t>
+          <t>1.4.1.1</t>
         </is>
       </c>
       <c r="J50" t="inlineStr">
         <is>
-          <t>PRESIDENTE PRUDENTE</t>
+          <t>TRANSPORTE</t>
         </is>
       </c>
       <c r="K50" t="inlineStr">
         <is>
-          <t>1.4.1 PRESIDENTE PRUDENTE</t>
+          <t>1.4.1.1 TRANSPORTE</t>
         </is>
       </c>
       <c r="L50" t="inlineStr">
@@ -7762,42 +7762,42 @@
       </c>
       <c r="D51" t="inlineStr">
         <is>
-          <t>DESPESA</t>
+          <t>TRANSMOVE GSL</t>
         </is>
       </c>
       <c r="E51" t="inlineStr">
         <is>
-          <t>1.4 DESPESA</t>
+          <t>1.4 TRANSMOVE GSL</t>
         </is>
       </c>
       <c r="F51" t="inlineStr">
         <is>
-          <t>1.4</t>
+          <t>1.4.1</t>
         </is>
       </c>
       <c r="G51" t="inlineStr">
         <is>
-          <t>TRANSMOVE GSL</t>
+          <t>PRESIDENTE PRUDENTE</t>
         </is>
       </c>
       <c r="H51" t="inlineStr">
         <is>
-          <t>1.4 TRANSMOVE GSL</t>
+          <t>1.4.1 PRESIDENTE PRUDENTE</t>
         </is>
       </c>
       <c r="I51" t="inlineStr">
         <is>
-          <t>1.4.1</t>
+          <t>1.4.1.1</t>
         </is>
       </c>
       <c r="J51" t="inlineStr">
         <is>
-          <t>PRESIDENTE PRUDENTE</t>
+          <t>TRANSPORTE</t>
         </is>
       </c>
       <c r="K51" t="inlineStr">
         <is>
-          <t>1.4.1 PRESIDENTE PRUDENTE</t>
+          <t>1.4.1.1 TRANSPORTE</t>
         </is>
       </c>
       <c r="L51" t="inlineStr">
@@ -7908,42 +7908,42 @@
       </c>
       <c r="D52" t="inlineStr">
         <is>
-          <t>DESPESA</t>
+          <t>TRANSMOVE GSL</t>
         </is>
       </c>
       <c r="E52" t="inlineStr">
         <is>
-          <t>1.4 DESPESA</t>
+          <t>1.4 TRANSMOVE GSL</t>
         </is>
       </c>
       <c r="F52" t="inlineStr">
         <is>
-          <t>1.4</t>
+          <t>1.4.1</t>
         </is>
       </c>
       <c r="G52" t="inlineStr">
         <is>
-          <t>TRANSMOVE GSL</t>
+          <t>PRESIDENTE PRUDENTE</t>
         </is>
       </c>
       <c r="H52" t="inlineStr">
         <is>
-          <t>1.4 TRANSMOVE GSL</t>
+          <t>1.4.1 PRESIDENTE PRUDENTE</t>
         </is>
       </c>
       <c r="I52" t="inlineStr">
         <is>
-          <t>1.4.1</t>
+          <t>1.4.1.1</t>
         </is>
       </c>
       <c r="J52" t="inlineStr">
         <is>
-          <t>PRESIDENTE PRUDENTE</t>
+          <t>TRANSPORTE</t>
         </is>
       </c>
       <c r="K52" t="inlineStr">
         <is>
-          <t>1.4.1 PRESIDENTE PRUDENTE</t>
+          <t>1.4.1.1 TRANSPORTE</t>
         </is>
       </c>
       <c r="L52" t="inlineStr">
@@ -8054,42 +8054,42 @@
       </c>
       <c r="D53" t="inlineStr">
         <is>
-          <t>DESPESA</t>
+          <t>TRANSMOVE GSL</t>
         </is>
       </c>
       <c r="E53" t="inlineStr">
         <is>
-          <t>1.4 DESPESA</t>
+          <t>1.4 TRANSMOVE GSL</t>
         </is>
       </c>
       <c r="F53" t="inlineStr">
         <is>
-          <t>1.4</t>
+          <t>1.4.1</t>
         </is>
       </c>
       <c r="G53" t="inlineStr">
         <is>
-          <t>TRANSMOVE GSL</t>
+          <t>PRESIDENTE PRUDENTE</t>
         </is>
       </c>
       <c r="H53" t="inlineStr">
         <is>
-          <t>1.4 TRANSMOVE GSL</t>
+          <t>1.4.1 PRESIDENTE PRUDENTE</t>
         </is>
       </c>
       <c r="I53" t="inlineStr">
         <is>
-          <t>1.4.1</t>
+          <t>1.4.1.1</t>
         </is>
       </c>
       <c r="J53" t="inlineStr">
         <is>
-          <t>PRESIDENTE PRUDENTE</t>
+          <t>TRANSPORTE</t>
         </is>
       </c>
       <c r="K53" t="inlineStr">
         <is>
-          <t>1.4.1 PRESIDENTE PRUDENTE</t>
+          <t>1.4.1.1 TRANSPORTE</t>
         </is>
       </c>
       <c r="L53" t="inlineStr">
@@ -8200,42 +8200,42 @@
       </c>
       <c r="D54" t="inlineStr">
         <is>
-          <t>DESPESA</t>
+          <t>TRANSMOVE GSL</t>
         </is>
       </c>
       <c r="E54" t="inlineStr">
         <is>
-          <t>1.4 DESPESA</t>
+          <t>1.4 TRANSMOVE GSL</t>
         </is>
       </c>
       <c r="F54" t="inlineStr">
         <is>
-          <t>1.4</t>
+          <t>1.4.1</t>
         </is>
       </c>
       <c r="G54" t="inlineStr">
         <is>
-          <t>TRANSMOVE GSL</t>
+          <t>PRESIDENTE PRUDENTE</t>
         </is>
       </c>
       <c r="H54" t="inlineStr">
         <is>
-          <t>1.4 TRANSMOVE GSL</t>
+          <t>1.4.1 PRESIDENTE PRUDENTE</t>
         </is>
       </c>
       <c r="I54" t="inlineStr">
         <is>
-          <t>1.4.1</t>
+          <t>1.4.1.1</t>
         </is>
       </c>
       <c r="J54" t="inlineStr">
         <is>
-          <t>PRESIDENTE PRUDENTE</t>
+          <t>TRANSPORTE</t>
         </is>
       </c>
       <c r="K54" t="inlineStr">
         <is>
-          <t>1.4.1 PRESIDENTE PRUDENTE</t>
+          <t>1.4.1.1 TRANSPORTE</t>
         </is>
       </c>
       <c r="L54" t="inlineStr">
@@ -8346,42 +8346,42 @@
       </c>
       <c r="D55" t="inlineStr">
         <is>
-          <t>DESPESA</t>
+          <t>TRANSMOVE GSL</t>
         </is>
       </c>
       <c r="E55" t="inlineStr">
         <is>
-          <t>1.4 DESPESA</t>
+          <t>1.4 TRANSMOVE GSL</t>
         </is>
       </c>
       <c r="F55" t="inlineStr">
         <is>
-          <t>1.4</t>
+          <t>1.4.1</t>
         </is>
       </c>
       <c r="G55" t="inlineStr">
         <is>
-          <t>TRANSMOVE GSL</t>
+          <t>PRESIDENTE PRUDENTE</t>
         </is>
       </c>
       <c r="H55" t="inlineStr">
         <is>
-          <t>1.4 TRANSMOVE GSL</t>
+          <t>1.4.1 PRESIDENTE PRUDENTE</t>
         </is>
       </c>
       <c r="I55" t="inlineStr">
         <is>
-          <t>1.4.1</t>
+          <t>1.4.1.1</t>
         </is>
       </c>
       <c r="J55" t="inlineStr">
         <is>
-          <t>PRESIDENTE PRUDENTE</t>
+          <t>TRANSPORTE</t>
         </is>
       </c>
       <c r="K55" t="inlineStr">
         <is>
-          <t>1.4.1 PRESIDENTE PRUDENTE</t>
+          <t>1.4.1.1 TRANSPORTE</t>
         </is>
       </c>
       <c r="L55" t="inlineStr">
@@ -8492,42 +8492,42 @@
       </c>
       <c r="D56" t="inlineStr">
         <is>
-          <t>DESPESA</t>
+          <t>TRANSMOVE GSL</t>
         </is>
       </c>
       <c r="E56" t="inlineStr">
         <is>
-          <t>1.4 DESPESA</t>
+          <t>1.4 TRANSMOVE GSL</t>
         </is>
       </c>
       <c r="F56" t="inlineStr">
         <is>
-          <t>1.4</t>
+          <t>1.4.1</t>
         </is>
       </c>
       <c r="G56" t="inlineStr">
         <is>
-          <t>TRANSMOVE GSL</t>
+          <t>PRESIDENTE PRUDENTE</t>
         </is>
       </c>
       <c r="H56" t="inlineStr">
         <is>
-          <t>1.4 TRANSMOVE GSL</t>
+          <t>1.4.1 PRESIDENTE PRUDENTE</t>
         </is>
       </c>
       <c r="I56" t="inlineStr">
         <is>
-          <t>1.4.1</t>
+          <t>1.4.1.1</t>
         </is>
       </c>
       <c r="J56" t="inlineStr">
         <is>
-          <t>PRESIDENTE PRUDENTE</t>
+          <t>TRANSPORTE</t>
         </is>
       </c>
       <c r="K56" t="inlineStr">
         <is>
-          <t>1.4.1 PRESIDENTE PRUDENTE</t>
+          <t>1.4.1.1 TRANSPORTE</t>
         </is>
       </c>
       <c r="L56" t="inlineStr">
@@ -8638,42 +8638,42 @@
       </c>
       <c r="D57" t="inlineStr">
         <is>
-          <t>DESPESA</t>
+          <t>TRANSMOVE GSL</t>
         </is>
       </c>
       <c r="E57" t="inlineStr">
         <is>
-          <t>1.4 DESPESA</t>
+          <t>1.4 TRANSMOVE GSL</t>
         </is>
       </c>
       <c r="F57" t="inlineStr">
         <is>
-          <t>1.4</t>
+          <t>1.4.1</t>
         </is>
       </c>
       <c r="G57" t="inlineStr">
         <is>
-          <t>TRANSMOVE GSL</t>
+          <t>PRESIDENTE PRUDENTE</t>
         </is>
       </c>
       <c r="H57" t="inlineStr">
         <is>
-          <t>1.4 TRANSMOVE GSL</t>
+          <t>1.4.1 PRESIDENTE PRUDENTE</t>
         </is>
       </c>
       <c r="I57" t="inlineStr">
         <is>
-          <t>1.4.1</t>
+          <t>1.4.1.1</t>
         </is>
       </c>
       <c r="J57" t="inlineStr">
         <is>
-          <t>PRESIDENTE PRUDENTE</t>
+          <t>TRANSPORTE</t>
         </is>
       </c>
       <c r="K57" t="inlineStr">
         <is>
-          <t>1.4.1 PRESIDENTE PRUDENTE</t>
+          <t>1.4.1.1 TRANSPORTE</t>
         </is>
       </c>
       <c r="L57" t="inlineStr">
@@ -8784,42 +8784,42 @@
       </c>
       <c r="D58" t="inlineStr">
         <is>
-          <t>DESPESA</t>
+          <t>TRANSMOVE GSL</t>
         </is>
       </c>
       <c r="E58" t="inlineStr">
         <is>
-          <t>1.4 DESPESA</t>
+          <t>1.4 TRANSMOVE GSL</t>
         </is>
       </c>
       <c r="F58" t="inlineStr">
         <is>
-          <t>1.4</t>
+          <t>1.4.1</t>
         </is>
       </c>
       <c r="G58" t="inlineStr">
         <is>
-          <t>TRANSMOVE GSL</t>
+          <t>PRESIDENTE PRUDENTE</t>
         </is>
       </c>
       <c r="H58" t="inlineStr">
         <is>
-          <t>1.4 TRANSMOVE GSL</t>
+          <t>1.4.1 PRESIDENTE PRUDENTE</t>
         </is>
       </c>
       <c r="I58" t="inlineStr">
         <is>
-          <t>1.4.1</t>
+          <t>1.4.1.1</t>
         </is>
       </c>
       <c r="J58" t="inlineStr">
         <is>
-          <t>PRESIDENTE PRUDENTE</t>
+          <t>TRANSPORTE</t>
         </is>
       </c>
       <c r="K58" t="inlineStr">
         <is>
-          <t>1.4.1 PRESIDENTE PRUDENTE</t>
+          <t>1.4.1.1 TRANSPORTE</t>
         </is>
       </c>
       <c r="L58" t="inlineStr">
@@ -8930,42 +8930,42 @@
       </c>
       <c r="D59" t="inlineStr">
         <is>
-          <t>DESPESA</t>
+          <t>TRANSMOVE GSL</t>
         </is>
       </c>
       <c r="E59" t="inlineStr">
         <is>
-          <t>1.4 DESPESA</t>
+          <t>1.4 TRANSMOVE GSL</t>
         </is>
       </c>
       <c r="F59" t="inlineStr">
         <is>
-          <t>1.4</t>
+          <t>1.4.1</t>
         </is>
       </c>
       <c r="G59" t="inlineStr">
         <is>
-          <t>TRANSMOVE GSL</t>
+          <t>PRESIDENTE PRUDENTE</t>
         </is>
       </c>
       <c r="H59" t="inlineStr">
         <is>
-          <t>1.4 TRANSMOVE GSL</t>
+          <t>1.4.1 PRESIDENTE PRUDENTE</t>
         </is>
       </c>
       <c r="I59" t="inlineStr">
         <is>
-          <t>1.4.1</t>
+          <t>1.4.1.1</t>
         </is>
       </c>
       <c r="J59" t="inlineStr">
         <is>
-          <t>PRESIDENTE PRUDENTE</t>
+          <t>TRANSPORTE</t>
         </is>
       </c>
       <c r="K59" t="inlineStr">
         <is>
-          <t>1.4.1 PRESIDENTE PRUDENTE</t>
+          <t>1.4.1.1 TRANSPORTE</t>
         </is>
       </c>
       <c r="L59" t="inlineStr">
@@ -9076,42 +9076,42 @@
       </c>
       <c r="D60" t="inlineStr">
         <is>
-          <t>DESPESA</t>
+          <t>TRANSMOVE GSL</t>
         </is>
       </c>
       <c r="E60" t="inlineStr">
         <is>
-          <t>1.4 DESPESA</t>
+          <t>1.4 TRANSMOVE GSL</t>
         </is>
       </c>
       <c r="F60" t="inlineStr">
         <is>
-          <t>1.4</t>
+          <t>1.4.1</t>
         </is>
       </c>
       <c r="G60" t="inlineStr">
         <is>
-          <t>TRANSMOVE GSL</t>
+          <t>PRESIDENTE PRUDENTE</t>
         </is>
       </c>
       <c r="H60" t="inlineStr">
         <is>
-          <t>1.4 TRANSMOVE GSL</t>
+          <t>1.4.1 PRESIDENTE PRUDENTE</t>
         </is>
       </c>
       <c r="I60" t="inlineStr">
         <is>
-          <t>1.4.1</t>
+          <t>1.4.1.1</t>
         </is>
       </c>
       <c r="J60" t="inlineStr">
         <is>
-          <t>PRESIDENTE PRUDENTE</t>
+          <t>TRANSPORTE</t>
         </is>
       </c>
       <c r="K60" t="inlineStr">
         <is>
-          <t>1.4.1 PRESIDENTE PRUDENTE</t>
+          <t>1.4.1.1 TRANSPORTE</t>
         </is>
       </c>
       <c r="L60" t="inlineStr">
@@ -9222,42 +9222,42 @@
       </c>
       <c r="D61" t="inlineStr">
         <is>
-          <t>DESPESA</t>
+          <t>TRANSMOVE GSL</t>
         </is>
       </c>
       <c r="E61" t="inlineStr">
         <is>
-          <t>1.4 DESPESA</t>
+          <t>1.4 TRANSMOVE GSL</t>
         </is>
       </c>
       <c r="F61" t="inlineStr">
         <is>
-          <t>1.4</t>
+          <t>1.4.1</t>
         </is>
       </c>
       <c r="G61" t="inlineStr">
         <is>
-          <t>TRANSMOVE GSL</t>
+          <t>PRESIDENTE PRUDENTE</t>
         </is>
       </c>
       <c r="H61" t="inlineStr">
         <is>
-          <t>1.4 TRANSMOVE GSL</t>
+          <t>1.4.1 PRESIDENTE PRUDENTE</t>
         </is>
       </c>
       <c r="I61" t="inlineStr">
         <is>
-          <t>1.4.1</t>
+          <t>1.4.1.1</t>
         </is>
       </c>
       <c r="J61" t="inlineStr">
         <is>
-          <t>PRESIDENTE PRUDENTE</t>
+          <t>TRANSPORTE</t>
         </is>
       </c>
       <c r="K61" t="inlineStr">
         <is>
-          <t>1.4.1 PRESIDENTE PRUDENTE</t>
+          <t>1.4.1.1 TRANSPORTE</t>
         </is>
       </c>
       <c r="L61" t="inlineStr">
@@ -9368,42 +9368,42 @@
       </c>
       <c r="D62" t="inlineStr">
         <is>
-          <t>DESPESA</t>
+          <t>TRANSMOVE GSL</t>
         </is>
       </c>
       <c r="E62" t="inlineStr">
         <is>
-          <t>1.4 DESPESA</t>
+          <t>1.4 TRANSMOVE GSL</t>
         </is>
       </c>
       <c r="F62" t="inlineStr">
         <is>
-          <t>1.4</t>
+          <t>1.4.1</t>
         </is>
       </c>
       <c r="G62" t="inlineStr">
         <is>
-          <t>TRANSMOVE GSL</t>
+          <t>PRESIDENTE PRUDENTE</t>
         </is>
       </c>
       <c r="H62" t="inlineStr">
         <is>
-          <t>1.4 TRANSMOVE GSL</t>
+          <t>1.4.1 PRESIDENTE PRUDENTE</t>
         </is>
       </c>
       <c r="I62" t="inlineStr">
         <is>
-          <t>1.4.1</t>
+          <t>1.4.1.1</t>
         </is>
       </c>
       <c r="J62" t="inlineStr">
         <is>
-          <t>PRESIDENTE PRUDENTE</t>
+          <t>TRANSPORTE</t>
         </is>
       </c>
       <c r="K62" t="inlineStr">
         <is>
-          <t>1.4.1 PRESIDENTE PRUDENTE</t>
+          <t>1.4.1.1 TRANSPORTE</t>
         </is>
       </c>
       <c r="L62" t="inlineStr">
@@ -9514,42 +9514,42 @@
       </c>
       <c r="D63" t="inlineStr">
         <is>
-          <t>DESPESA</t>
+          <t>TRANSMOVE GSL</t>
         </is>
       </c>
       <c r="E63" t="inlineStr">
         <is>
-          <t>1.4 DESPESA</t>
+          <t>1.4 TRANSMOVE GSL</t>
         </is>
       </c>
       <c r="F63" t="inlineStr">
         <is>
-          <t>1.4</t>
+          <t>1.4.1</t>
         </is>
       </c>
       <c r="G63" t="inlineStr">
         <is>
-          <t>TRANSMOVE GSL</t>
+          <t>PRESIDENTE PRUDENTE</t>
         </is>
       </c>
       <c r="H63" t="inlineStr">
         <is>
-          <t>1.4 TRANSMOVE GSL</t>
+          <t>1.4.1 PRESIDENTE PRUDENTE</t>
         </is>
       </c>
       <c r="I63" t="inlineStr">
         <is>
-          <t>1.4.1</t>
+          <t>1.4.1.1</t>
         </is>
       </c>
       <c r="J63" t="inlineStr">
         <is>
-          <t>PRESIDENTE PRUDENTE</t>
+          <t>TRANSPORTE</t>
         </is>
       </c>
       <c r="K63" t="inlineStr">
         <is>
-          <t>1.4.1 PRESIDENTE PRUDENTE</t>
+          <t>1.4.1.1 TRANSPORTE</t>
         </is>
       </c>
       <c r="L63" t="inlineStr">
@@ -9660,42 +9660,42 @@
       </c>
       <c r="D64" t="inlineStr">
         <is>
-          <t>DESPESA</t>
+          <t>TRANSMOVE GSL</t>
         </is>
       </c>
       <c r="E64" t="inlineStr">
         <is>
-          <t>1.4 DESPESA</t>
+          <t>1.4 TRANSMOVE GSL</t>
         </is>
       </c>
       <c r="F64" t="inlineStr">
         <is>
-          <t>1.4</t>
+          <t>1.4.1</t>
         </is>
       </c>
       <c r="G64" t="inlineStr">
         <is>
-          <t>TRANSMOVE GSL</t>
+          <t>PRESIDENTE PRUDENTE</t>
         </is>
       </c>
       <c r="H64" t="inlineStr">
         <is>
-          <t>1.4 TRANSMOVE GSL</t>
+          <t>1.4.1 PRESIDENTE PRUDENTE</t>
         </is>
       </c>
       <c r="I64" t="inlineStr">
         <is>
-          <t>1.4.1</t>
+          <t>1.4.1.1</t>
         </is>
       </c>
       <c r="J64" t="inlineStr">
         <is>
-          <t>PRESIDENTE PRUDENTE</t>
+          <t>TRANSPORTE</t>
         </is>
       </c>
       <c r="K64" t="inlineStr">
         <is>
-          <t>1.4.1 PRESIDENTE PRUDENTE</t>
+          <t>1.4.1.1 TRANSPORTE</t>
         </is>
       </c>
       <c r="L64" t="inlineStr">
@@ -9806,42 +9806,42 @@
       </c>
       <c r="D65" t="inlineStr">
         <is>
-          <t>DESPESA</t>
+          <t>TRANSMOVE GSL</t>
         </is>
       </c>
       <c r="E65" t="inlineStr">
         <is>
-          <t>1.4 DESPESA</t>
+          <t>1.4 TRANSMOVE GSL</t>
         </is>
       </c>
       <c r="F65" t="inlineStr">
         <is>
-          <t>1.4</t>
+          <t>1.4.1</t>
         </is>
       </c>
       <c r="G65" t="inlineStr">
         <is>
-          <t>TRANSMOVE GSL</t>
+          <t>PRESIDENTE PRUDENTE</t>
         </is>
       </c>
       <c r="H65" t="inlineStr">
         <is>
-          <t>1.4 TRANSMOVE GSL</t>
+          <t>1.4.1 PRESIDENTE PRUDENTE</t>
         </is>
       </c>
       <c r="I65" t="inlineStr">
         <is>
-          <t>1.4.1</t>
+          <t>1.4.1.1</t>
         </is>
       </c>
       <c r="J65" t="inlineStr">
         <is>
-          <t>PRESIDENTE PRUDENTE</t>
+          <t>TRANSPORTE</t>
         </is>
       </c>
       <c r="K65" t="inlineStr">
         <is>
-          <t>1.4.1 PRESIDENTE PRUDENTE</t>
+          <t>1.4.1.1 TRANSPORTE</t>
         </is>
       </c>
       <c r="L65" t="inlineStr">
@@ -9952,42 +9952,42 @@
       </c>
       <c r="D66" t="inlineStr">
         <is>
-          <t>DESPESA</t>
+          <t>TRANSMOVE GSL</t>
         </is>
       </c>
       <c r="E66" t="inlineStr">
         <is>
-          <t>1.4 DESPESA</t>
+          <t>1.4 TRANSMOVE GSL</t>
         </is>
       </c>
       <c r="F66" t="inlineStr">
         <is>
-          <t>1.4</t>
+          <t>1.4.1</t>
         </is>
       </c>
       <c r="G66" t="inlineStr">
         <is>
-          <t>TRANSMOVE GSL</t>
+          <t>PRESIDENTE PRUDENTE</t>
         </is>
       </c>
       <c r="H66" t="inlineStr">
         <is>
-          <t>1.4 TRANSMOVE GSL</t>
+          <t>1.4.1 PRESIDENTE PRUDENTE</t>
         </is>
       </c>
       <c r="I66" t="inlineStr">
         <is>
-          <t>1.4.1</t>
+          <t>1.4.1.1</t>
         </is>
       </c>
       <c r="J66" t="inlineStr">
         <is>
-          <t>PRESIDENTE PRUDENTE</t>
+          <t>TRANSPORTE</t>
         </is>
       </c>
       <c r="K66" t="inlineStr">
         <is>
-          <t>1.4.1 PRESIDENTE PRUDENTE</t>
+          <t>1.4.1.1 TRANSPORTE</t>
         </is>
       </c>
       <c r="L66" t="inlineStr">
@@ -10098,42 +10098,42 @@
       </c>
       <c r="D67" t="inlineStr">
         <is>
-          <t>DESPESA</t>
+          <t>TRANSMOVE GSL</t>
         </is>
       </c>
       <c r="E67" t="inlineStr">
         <is>
-          <t>1.4 DESPESA</t>
+          <t>1.4 TRANSMOVE GSL</t>
         </is>
       </c>
       <c r="F67" t="inlineStr">
         <is>
-          <t>1.4</t>
+          <t>1.4.1</t>
         </is>
       </c>
       <c r="G67" t="inlineStr">
         <is>
-          <t>TRANSMOVE GSL</t>
+          <t>PRESIDENTE PRUDENTE</t>
         </is>
       </c>
       <c r="H67" t="inlineStr">
         <is>
-          <t>1.4 TRANSMOVE GSL</t>
+          <t>1.4.1 PRESIDENTE PRUDENTE</t>
         </is>
       </c>
       <c r="I67" t="inlineStr">
         <is>
-          <t>1.4.1</t>
+          <t>1.4.1.1</t>
         </is>
       </c>
       <c r="J67" t="inlineStr">
         <is>
-          <t>PRESIDENTE PRUDENTE</t>
+          <t>TRANSPORTE</t>
         </is>
       </c>
       <c r="K67" t="inlineStr">
         <is>
-          <t>1.4.1 PRESIDENTE PRUDENTE</t>
+          <t>1.4.1.1 TRANSPORTE</t>
         </is>
       </c>
       <c r="L67" t="inlineStr">
@@ -10244,42 +10244,42 @@
       </c>
       <c r="D68" t="inlineStr">
         <is>
-          <t>DESPESA</t>
+          <t>TRANSMOVE GSL</t>
         </is>
       </c>
       <c r="E68" t="inlineStr">
         <is>
-          <t>1.4 DESPESA</t>
+          <t>1.4 TRANSMOVE GSL</t>
         </is>
       </c>
       <c r="F68" t="inlineStr">
         <is>
-          <t>1.4</t>
+          <t>1.4.1</t>
         </is>
       </c>
       <c r="G68" t="inlineStr">
         <is>
-          <t>TRANSMOVE GSL</t>
+          <t>PRESIDENTE PRUDENTE</t>
         </is>
       </c>
       <c r="H68" t="inlineStr">
         <is>
-          <t>1.4 TRANSMOVE GSL</t>
+          <t>1.4.1 PRESIDENTE PRUDENTE</t>
         </is>
       </c>
       <c r="I68" t="inlineStr">
         <is>
-          <t>1.4.1</t>
+          <t>1.4.1.1</t>
         </is>
       </c>
       <c r="J68" t="inlineStr">
         <is>
-          <t>PRESIDENTE PRUDENTE</t>
+          <t>TRANSPORTE</t>
         </is>
       </c>
       <c r="K68" t="inlineStr">
         <is>
-          <t>1.4.1 PRESIDENTE PRUDENTE</t>
+          <t>1.4.1.1 TRANSPORTE</t>
         </is>
       </c>
       <c r="L68" t="inlineStr">
@@ -10390,42 +10390,42 @@
       </c>
       <c r="D69" t="inlineStr">
         <is>
-          <t>DESPESA</t>
+          <t>TRANSMOVE GSL</t>
         </is>
       </c>
       <c r="E69" t="inlineStr">
         <is>
-          <t>1.4 DESPESA</t>
+          <t>1.4 TRANSMOVE GSL</t>
         </is>
       </c>
       <c r="F69" t="inlineStr">
         <is>
-          <t>1.4</t>
+          <t>1.4.1</t>
         </is>
       </c>
       <c r="G69" t="inlineStr">
         <is>
-          <t>TRANSMOVE GSL</t>
+          <t>PRESIDENTE PRUDENTE</t>
         </is>
       </c>
       <c r="H69" t="inlineStr">
         <is>
-          <t>1.4 TRANSMOVE GSL</t>
+          <t>1.4.1 PRESIDENTE PRUDENTE</t>
         </is>
       </c>
       <c r="I69" t="inlineStr">
         <is>
-          <t>1.4.1</t>
+          <t>1.4.1.1</t>
         </is>
       </c>
       <c r="J69" t="inlineStr">
         <is>
-          <t>PRESIDENTE PRUDENTE</t>
+          <t>TRANSPORTE</t>
         </is>
       </c>
       <c r="K69" t="inlineStr">
         <is>
-          <t>1.4.1 PRESIDENTE PRUDENTE</t>
+          <t>1.4.1.1 TRANSPORTE</t>
         </is>
       </c>
       <c r="L69" t="inlineStr">

</xml_diff>